<commit_message>
Barefoot: confirmed mast/cabinet costs in the risk model; client-facing detailed cost schedule at R335,000 with monthly costs and payment options
Co-Authored-By: Claude Fable 5.1 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01F75G8iv8ooxhkGc1PV5mNB
</commit_message>
<xml_diff>
--- a/proposals/Barefoot_Build_Risk_Model_2026-09-29.xlsx
+++ b/proposals/Barefoot_Build_Risk_Model_2026-09-29.xlsx
@@ -625,11 +625,11 @@
         </is>
       </c>
       <c r="B6" s="6" t="n">
-        <v>305000</v>
+        <v>335000</v>
       </c>
       <c r="C6" s="2" t="inlineStr">
         <is>
-          <t>Challenged floor from the 29 Sep memo. Change to test other prices (355,000 = as proposed).</t>
+          <t>29 Sep: client schedule generated at R335,000 (15.2% GP at current inputs). Change to test.</t>
         </is>
       </c>
     </row>
@@ -749,6 +749,7 @@
       </c>
       <c r="C14" s="2" t="inlineStr"/>
     </row>
+    <row r="15"/>
     <row r="16">
       <c r="A16" s="3" t="inlineStr">
         <is>
@@ -981,6 +982,7 @@
         </is>
       </c>
     </row>
+    <row r="32"/>
     <row r="33">
       <c r="A33" s="3" t="inlineStr">
         <is>
@@ -1159,12 +1161,12 @@
           <t>Outdoor cabinet, bare (CTTX stock)</t>
         </is>
       </c>
-      <c r="B45" s="7" t="n">
-        <v>10000</v>
+      <c r="B45" s="6" t="n">
+        <v>8000</v>
       </c>
       <c r="C45" s="2" t="inlineStr">
         <is>
-          <t>TBC — Gerhard. Was R28,670 fully fitted with MPPT/battery/switchgear.</t>
+          <t>Gerhard, 29 Sep: floor R8,000 - confirmed</t>
         </is>
       </c>
     </row>
@@ -1174,12 +1176,12 @@
           <t>6m mast with plinth, installed (CTTX stock)</t>
         </is>
       </c>
-      <c r="B46" s="7" t="n">
-        <v>25000</v>
+      <c r="B46" s="6" t="n">
+        <v>22000</v>
       </c>
       <c r="C46" s="2" t="inlineStr">
         <is>
-          <t>TBC — Gerhard</t>
+          <t>Gerhard, 29 Sep: floor R22,000 - confirmed</t>
         </is>
       </c>
     </row>
@@ -2173,11 +2175,11 @@
     <row r="6">
       <c r="A6" s="4" t="inlineStr">
         <is>
-          <t>6m mast cost estimate wrong (R25k assumed)</t>
+          <t>6m mast cost - CONFIRMED R22,000 (Gerhard 29 Sep)</t>
         </is>
       </c>
       <c r="B6" s="30" t="n">
-        <v>0.5</v>
+        <v>0</v>
       </c>
       <c r="C6" s="13">
         <f>5000</f>
@@ -2194,18 +2196,18 @@
       </c>
       <c r="F6" s="14" t="inlineStr">
         <is>
-          <t>OPEN</t>
+          <t>CLOSED</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" s="4" t="inlineStr">
         <is>
-          <t>Bare cabinet cost estimate wrong (R10k assumed)</t>
+          <t>Bare cabinet cost - CONFIRMED R8,000 (Gerhard 29 Sep)</t>
         </is>
       </c>
       <c r="B7" s="30" t="n">
-        <v>0.5</v>
+        <v>0</v>
       </c>
       <c r="C7" s="13">
         <f>4000</f>
@@ -2222,7 +2224,7 @@
       </c>
       <c r="F7" s="14" t="inlineStr">
         <is>
-          <t>OPEN</t>
+          <t>CLOSED</t>
         </is>
       </c>
     </row>
@@ -2534,6 +2536,7 @@
         </is>
       </c>
     </row>
+    <row r="19"/>
     <row r="20">
       <c r="A20" s="31" t="inlineStr">
         <is>
@@ -2556,6 +2559,7 @@
         <v/>
       </c>
     </row>
+    <row r="22"/>
     <row r="23">
       <c r="A23" s="24" t="inlineStr">
         <is>
@@ -2589,6 +2593,7 @@
         <v/>
       </c>
     </row>
+    <row r="26"/>
     <row r="27" ht="45" customHeight="1">
       <c r="A27" s="2" t="inlineStr">
         <is>

</xml_diff>

<commit_message>
Barefoot risk model: mast LOS risk reduced after Gerhard's on-site sighting of Olifants Nek
Co-Authored-By: Claude Fable 5.1 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01F75G8iv8ooxhkGc1PV5mNB
</commit_message>
<xml_diff>
--- a/proposals/Barefoot_Build_Risk_Model_2026-09-29.xlsx
+++ b/proposals/Barefoot_Build_Risk_Model_2026-09-29.xlsx
@@ -749,7 +749,6 @@
       </c>
       <c r="C14" s="2" t="inlineStr"/>
     </row>
-    <row r="15"/>
     <row r="16">
       <c r="A16" s="3" t="inlineStr">
         <is>
@@ -982,7 +981,6 @@
         </is>
       </c>
     </row>
-    <row r="32"/>
     <row r="33">
       <c r="A33" s="3" t="inlineStr">
         <is>
@@ -2147,11 +2145,11 @@
     <row r="5">
       <c r="A5" s="4" t="inlineStr">
         <is>
-          <t>Mast: 6m has no LOS to Olifants Nek or the staff village → build 9m</t>
+          <t>Mast: 6m has no usable LOS → build 9m. Gerhard stood at the mast position 29 Sep and saw clear LOS to Olifants Nek at ground level; Vodacom's own confirmation at 6m and Abel's 3 km staff-village LOS remain.</t>
         </is>
       </c>
       <c r="B5" s="30" t="n">
-        <v>0.4</v>
+        <v>0.15</v>
       </c>
       <c r="C5" s="13">
         <f>'1. Inputs'!$B$47-IF('1. Inputs'!$B$27=9,'1. Inputs'!$B$47,'1. Inputs'!$B$46)</f>
@@ -2163,12 +2161,12 @@
       </c>
       <c r="E5" s="2" t="inlineStr">
         <is>
-          <t>Duane desktop feasibility at 6m (asked 29 Sep); Abel LOS from survey</t>
+          <t>Vodacom desktop confirmation (Duane, asked 29 Sep); Abel: staff village LOS at 6m</t>
         </is>
       </c>
       <c r="F5" s="14" t="inlineStr">
         <is>
-          <t>OPEN</t>
+          <t>REDUCED</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Barefoot: installation planned at 4 days; client schedule regenerated (reusable generator)
Co-Authored-By: Claude Fable 5.1 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01F75G8iv8ooxhkGc1PV5mNB
</commit_message>
<xml_diff>
--- a/proposals/Barefoot_Build_Risk_Model_2026-09-29.xlsx
+++ b/proposals/Barefoot_Build_Risk_Model_2026-09-29.xlsx
@@ -749,6 +749,7 @@
       </c>
       <c r="C14" s="2" t="inlineStr"/>
     </row>
+    <row r="15"/>
     <row r="16">
       <c r="A16" s="3" t="inlineStr">
         <is>
@@ -943,11 +944,11 @@
         </is>
       </c>
       <c r="B29" s="8" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="C29" s="2" t="inlineStr">
         <is>
-          <t>25 Sep quote; 25 sites over 3 days = 8/day — tight. See risk register.</t>
+          <t>Gerhard, 29 Sep: 4 days for 25–28 radios (was 3)</t>
         </is>
       </c>
     </row>
@@ -981,6 +982,7 @@
         </is>
       </c>
     </row>
+    <row r="32"/>
     <row r="33">
       <c r="A33" s="3" t="inlineStr">
         <is>
@@ -2313,14 +2315,14 @@
     <row r="11">
       <c r="A11" s="4" t="inlineStr">
         <is>
-          <t>Installation overruns by 2 days (25 sites in 3 days = 8/day)</t>
+          <t>Installation overruns by 1 day beyond the planned 4</t>
         </is>
       </c>
       <c r="B11" s="30" t="n">
-        <v>0.5</v>
+        <v>0.25</v>
       </c>
       <c r="C11" s="13">
-        <f>2*'1. Inputs'!$B$52</f>
+        <f>1*'1. Inputs'!$B$52</f>
         <v/>
       </c>
       <c r="D11" s="13">
@@ -2334,7 +2336,7 @@
       </c>
       <c r="F11" s="14" t="inlineStr">
         <is>
-          <t>OPEN</t>
+          <t>REDUCED</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Barefoot: Olifants Nek is 3rd-party — Vodacom minimum is BC 300 Mbps at R6,510.46 cost; schedule, model and memo recalculated
Co-Authored-By: Claude Fable 5.1 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01F75G8iv8ooxhkGc1PV5mNB
</commit_message>
<xml_diff>
--- a/proposals/Barefoot_Build_Risk_Model_2026-09-29.xlsx
+++ b/proposals/Barefoot_Build_Risk_Model_2026-09-29.xlsx
@@ -636,15 +636,15 @@
     <row r="7">
       <c r="A7" s="4" t="inlineStr">
         <is>
-          <t>Vodacom BC 100 Mbps 36m — CTTX cost / month</t>
+          <t>Vodacom BC 300 Mbps 36m — CTTX cost / month (minimum service at Olifants Nek)</t>
         </is>
       </c>
       <c r="B7" s="6" t="n">
-        <v>4152.04</v>
+        <v>6510.46</v>
       </c>
       <c r="C7" s="2" t="inlineStr">
         <is>
-          <t>Fixed Services AAG 092026 (Duane, 14 Sep 2026)</t>
+          <t>Duane Forlee, 1 Oct 2026: EAS feedback — distance + Telkom 3rd-party; BC 300 is the minimum service. 'Based on the old costing to meet the rand value criteria.'</t>
         </is>
       </c>
     </row>
@@ -674,7 +674,7 @@
       </c>
       <c r="C9" s="2" t="inlineStr">
         <is>
-          <t>AAG: '3rd-party infrastructure will incur additional cost'. Olifants Nek = Telkom site. Asked Duane 29 Sep.</t>
+          <t>Resolved 1 Oct: surcharge is embedded in the BC300 rate above</t>
         </is>
       </c>
     </row>
@@ -2483,11 +2483,11 @@
     <row r="17">
       <c r="A17" s="4" t="inlineStr">
         <is>
-          <t>Vodacom 3rd-party surcharge at Olifants Nek — CTTX absorbs it for the 36-month term rather than re-open the price</t>
+          <t>Vodacom 3rd-party surcharge — RESOLVED 1 Oct: BC300 minimum at R6,510.46 cost; priced into the MRC</t>
         </is>
       </c>
       <c r="B17" s="30" t="n">
-        <v>0.3</v>
+        <v>0</v>
       </c>
       <c r="C17" s="13">
         <f>36*500</f>
@@ -2504,7 +2504,7 @@
       </c>
       <c r="F17" s="14" t="inlineStr">
         <is>
-          <t>OPEN</t>
+          <t>CLOSED</t>
         </is>
       </c>
     </row>

</xml_diff>